<commit_message>
updates to omop part to move away from clinical relevance and add specialty plot
</commit_message>
<xml_diff>
--- a/OMOP Analysis/Results/Cohort/Output_gt_overall_healthcare_roles_count_OMOP.xlsx
+++ b/OMOP Analysis/Results/Cohort/Output_gt_overall_healthcare_roles_count_OMOP.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -376,19 +376,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Administrative Non-clinical</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>327,342 (37.3%)</t>
+          <t>327,106 (37.3%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General Practitioner</t>
+          <t>GP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -400,12 +400,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Non-registered other</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>107,565 (12.3%)</t>
+          <t>121,461 (13.8%)</t>
         </is>
       </c>
     </row>
@@ -417,7 +417,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>85,458 (9.7%)</t>
+          <t>42,557 (4.9%)</t>
         </is>
       </c>
     </row>
@@ -436,401 +436,449 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>__Healthcare Provider Roles__</t>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>22,347 (2.5%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>General Practice</t>
+          <t>AHP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>325,922 (37.2%)</t>
+          <t>6,651 (0.8%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Other Technician</t>
+          <t>Medic non-GP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>118,097 (13.5%)</t>
+          <t>236 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Registered Record Administrator</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>107,810 (12.3%)</t>
+          <t>7 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Case Manager / Care Coordinator</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>76,318 (8.7%)</t>
+          <t>__Healthcare Provider Roles__</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Community Health Nurse Practitioner</t>
+          <t>General Practice</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>42,901 (4.9%)</t>
+          <t>325,922 (37.2%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Medical Physician Assistant</t>
+          <t>Other Technician</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>36,677 (4.2%)</t>
+          <t>118,097 (13.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>No matching concept</t>
+          <t>Registered Record Administrator</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>31,006 (3.5%)</t>
+          <t>107,810 (12.3%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Physician Assistant</t>
+          <t>Case Manager / Care Coordinator</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,368 (3.2%)</t>
+          <t>76,318 (8.7%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Community Health Worker</t>
+          <t>Community Health Nurse Practitioner</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>22,347 (2.5%)</t>
+          <t>42,901 (4.9%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Health Information Technician</t>
+          <t>Medical Physician Assistant</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>20,920 (2.4%)</t>
+          <t>36,677 (4.2%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Registered Community Health Nurse</t>
+          <t>No matching concept</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15,197 (1.7%)</t>
+          <t>31,006 (3.5%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Clinical Nurse Specialist</t>
+          <t>Physician Assistant</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11,862 (1.4%)</t>
+          <t>28,368 (3.2%)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Registered Nurse</t>
+          <t>Community Health Worker</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9,644 (1.1%)</t>
+          <t>22,347 (2.5%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Phlebotomist</t>
+          <t>Health Information Technician</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>6,136 (0.7%)</t>
+          <t>20,920 (2.4%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pharmacy Technician</t>
+          <t>Registered Community Health Nurse</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>6,094 (0.7%)</t>
+          <t>15,197 (1.7%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pharmacist</t>
+          <t>Clinical Nurse Specialist</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>5,488 (0.6%)</t>
+          <t>11,862 (1.4%)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Physician Office Based Coding Specialist</t>
+          <t>Registered Nurse</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3,961 (0.5%)</t>
+          <t>9,644 (1.1%)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Registered General Practice Nurse</t>
+          <t>Phlebotomist</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>3,848 (0.4%)</t>
+          <t>6,136 (0.7%)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nurse Practitioner</t>
+          <t>Pharmacy Technician</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1,916 (0.2%)</t>
+          <t>6,094 (0.7%)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Specialist</t>
+          <t>Pharmacist</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>593 (0.1%)</t>
+          <t>5,488 (0.6%)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Surgical Physician Assistant</t>
+          <t>Physician Office Based Coding Specialist</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>543 (0.1%)</t>
+          <t>3,961 (0.5%)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Physical Hand Therapist</t>
+          <t>Registered General Practice Nurse</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>468 (0.1%)</t>
+          <t>3,848 (0.4%)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Paramedic</t>
+          <t>Nurse Practitioner</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>426 (0.0%)</t>
+          <t>1,916 (0.2%)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Specialist</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>236 (0.0%)</t>
+          <t>593 (0.1%)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Professional Behavioral Health Counselor</t>
+          <t>Surgical Physician Assistant</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>141 (0.0%)</t>
+          <t>543 (0.1%)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Podiatrist</t>
+          <t>Physical Hand Therapist</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>112 (0.0%)</t>
+          <t>468 (0.1%)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Community Psych / Mental Health Nurse</t>
+          <t>Paramedic</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>90 (0.0%)</t>
+          <t>426 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Registered Dietitian</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>75 (0.0%)</t>
+          <t>236 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marriage and Family Therapist</t>
+          <t>Professional Behavioral Health Counselor</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>51 (0.0%)</t>
+          <t>141 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Radiography Technologist</t>
+          <t>Podiatrist</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28 (0.0%)</t>
+          <t>112 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Behavioral Health &amp; Social Service Providers, Psychologist, Clinical</t>
+          <t>Community Psych / Mental Health Nurse</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>8 (0.0%)</t>
+          <t>90 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Social Worker</t>
+          <t>Registered Dietitian</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>7 (0.0%)</t>
+          <t>75 (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>Marriage and Family Therapist</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>51 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Radiography Technologist</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>28 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Behavioral Health &amp; Social Service Providers, Psychologist, Clinical</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>8 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Social Worker</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>7 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Midwife</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>3 (0.0%)</t>
         </is>

</xml_diff>